<commit_message>
fix(problem-bank): 관계대명사 what 문항의 O/X 정답 오류
`What he need is money.` 를 비롯해 14~18번 다섯 문항이 전부 `he need`로 적혀
있었다. 관계절 안의 주어가 `he`라 `needs`가 맞는데, 앞의 세 문항은 그대로
**O(정문)** 으로 표시돼 있어 틀린 문법을 가르치고 있었다. 같은 세트의 26번
`What he did were wrong.`은 단수 규칙을 적용해 X로 처리하고 있어 서로 모순이었다.

O/X 라벨은 그대로 두고 `need` → `needs`만 고쳤다. 라벨을 뒤집으면 17번의
「the thing what은 틀렸다」·18번의 「That이 아니라 What」이라는 원래 출제
의도가 깨진다.

엑셀 원본부터 고치고 임포트 스크립트로 JSON을 재생성했다 — JSON만 손보면
다음 임포트 때 되돌아온다. 재생성 결과 diff는 15줄(5문항 × 3학년 사본)뿐이다.

임포트 스크립트가 학생 리포를 형제 폴더로 가정해 음성 갱신을 조용히 건너뛰고
있던 것도 같이 고쳤다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/problem-bank-import.xlsx
+++ b/scripts/problem-bank-import.xlsx
@@ -152,7 +152,7 @@
     <t>당신이 기르는  애완동물들조차도  당신이  어떤 종류의  사람인지를  어느 정도 보여줍니다.</t>
   </si>
   <si>
-    <t>What he need is money.</t>
+    <t>What he needs is money.</t>
   </si>
   <si>
     <t>기르다</t>
@@ -206,7 +206,7 @@
     <t>이런 검사들  중 하나는  DAPR 검사입니다.</t>
   </si>
   <si>
-    <t>The thing which he need is money.</t>
+    <t>The thing which he needs is money.</t>
   </si>
   <si>
     <t>somehow</t>
@@ -239,7 +239,7 @@
     <t>기초단어 여부</t>
   </si>
   <si>
-    <t>The thing that he need is money.</t>
+    <t>The thing that he needs is money.</t>
   </si>
   <si>
     <t>심지어</t>
@@ -251,7 +251,7 @@
     <t>be related to</t>
   </si>
   <si>
-    <t>The thing what he need is money.</t>
+    <t>The thing what he needs is money.</t>
   </si>
   <si>
     <t>~와 관련있다</t>
@@ -308,7 +308,7 @@
     <t>의사들은 다양한 그림 그리기 검사를 사용해 오고 있습니다.</t>
   </si>
   <si>
-    <t>That he need is money.</t>
+    <t>That he needs is money.</t>
   </si>
   <si>
     <t>study</t>

</xml_diff>